<commit_message>
Dealer list: rep name (Sales_Rep_Name__c read for dealer + rep, list column) and updatedAt (LastModifiedDate cache column)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Sundial_Customer__c_Field_Design.xlsx
+++ b/docs/Sundial_Customer__c_Field_Design.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2709" uniqueCount="867">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2716" uniqueCount="870">
   <si>
     <t>Sundial Section</t>
   </si>
@@ -2615,6 +2615,15 @@
   </si>
   <si>
     <t>Appointment setter</t>
+  </si>
+  <si>
+    <t>Sales Rep Name</t>
+  </si>
+  <si>
+    <t>Sales_Rep_Name__c</t>
+  </si>
+  <si>
+    <t>The Sales Rep's name, set automatically. For list rows (the dealer list); the record page shows Sales Rep.</t>
   </si>
 </sst>
 </file>
@@ -3013,7 +3022,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H340"/>
+  <dimension ref="A1:H341"/>
   <sheetFormatPr defaultRowHeight="15.75" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.5" customHeight="1"/>
   <cols>
     <col min="1" max="2" width="30.875" style="1" customWidth="1"/>
@@ -11839,6 +11848,30 @@
         <v>14</v>
       </c>
     </row>
+    <row r="341" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A341" s="1" t="s">
+        <v>834</v>
+      </c>
+      <c r="B341" s="1" t="s">
+        <v>867</v>
+      </c>
+      <c r="C341" s="1" t="s">
+        <v>868</v>
+      </c>
+      <c r="D341" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="E341" s="1" t="s">
+        <v>869</v>
+      </c>
+      <c r="F341" s="1"/>
+      <c r="G341" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="H341" s="1" t="s">
+        <v>146</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Dealer feedback 1: fold Permitting Received into Permit Submitted; hide permit dates and NS adder cost basis
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Sundial_Customer__c_Field_Design.xlsx
+++ b/docs/Sundial_Customer__c_Field_Design.xlsx
@@ -10721,7 +10721,7 @@
         <v>14</v>
       </c>
       <c r="H296" s="1" t="s">
-        <v>146</v>
+        <v>14</v>
       </c>
     </row>
     <row r="297" spans="1:8" x14ac:dyDescent="0.25">
@@ -10747,7 +10747,7 @@
         <v>14</v>
       </c>
       <c r="H297" s="1" t="s">
-        <v>146</v>
+        <v>14</v>
       </c>
     </row>
     <row r="298" spans="1:8" x14ac:dyDescent="0.25">
@@ -10773,7 +10773,7 @@
         <v>14</v>
       </c>
       <c r="H298" s="1" t="s">
-        <v>146</v>
+        <v>14</v>
       </c>
     </row>
     <row r="299" spans="1:8" x14ac:dyDescent="0.25">
@@ -10847,7 +10847,7 @@
         <v>14</v>
       </c>
       <c r="H301" s="1" t="s">
-        <v>146</v>
+        <v>14</v>
       </c>
     </row>
     <row r="302" spans="1:8" x14ac:dyDescent="0.25">
@@ -10873,7 +10873,7 @@
         <v>14</v>
       </c>
       <c r="H302" s="1" t="s">
-        <v>146</v>
+        <v>14</v>
       </c>
     </row>
     <row r="303" spans="1:8" x14ac:dyDescent="0.25">
@@ -10899,7 +10899,7 @@
         <v>14</v>
       </c>
       <c r="H303" s="1" t="s">
-        <v>146</v>
+        <v>14</v>
       </c>
     </row>
     <row r="304" spans="1:8" x14ac:dyDescent="0.25">
@@ -10973,7 +10973,7 @@
         <v>14</v>
       </c>
       <c r="H306" s="1" t="s">
-        <v>146</v>
+        <v>14</v>
       </c>
     </row>
     <row r="307" spans="1:8" x14ac:dyDescent="0.25">
@@ -10999,7 +10999,7 @@
         <v>14</v>
       </c>
       <c r="H307" s="1" t="s">
-        <v>146</v>
+        <v>14</v>
       </c>
     </row>
     <row r="308" spans="1:8" x14ac:dyDescent="0.25">
@@ -11025,7 +11025,7 @@
         <v>14</v>
       </c>
       <c r="H308" s="1" t="s">
-        <v>146</v>
+        <v>14</v>
       </c>
     </row>
     <row r="309" spans="1:8" x14ac:dyDescent="0.25">
@@ -11099,7 +11099,7 @@
         <v>14</v>
       </c>
       <c r="H311" s="1" t="s">
-        <v>146</v>
+        <v>14</v>
       </c>
     </row>
     <row r="312" spans="1:8" x14ac:dyDescent="0.25">
@@ -11125,7 +11125,7 @@
         <v>14</v>
       </c>
       <c r="H312" s="1" t="s">
-        <v>146</v>
+        <v>14</v>
       </c>
     </row>
     <row r="313" spans="1:8" x14ac:dyDescent="0.25">
@@ -11151,7 +11151,7 @@
         <v>14</v>
       </c>
       <c r="H313" s="1" t="s">
-        <v>146</v>
+        <v>14</v>
       </c>
     </row>
     <row r="314" spans="1:8" x14ac:dyDescent="0.25">
@@ -11225,7 +11225,7 @@
         <v>14</v>
       </c>
       <c r="H316" s="1" t="s">
-        <v>146</v>
+        <v>14</v>
       </c>
     </row>
     <row r="317" spans="1:8" x14ac:dyDescent="0.25">
@@ -11251,7 +11251,7 @@
         <v>14</v>
       </c>
       <c r="H317" s="1" t="s">
-        <v>146</v>
+        <v>14</v>
       </c>
     </row>
     <row r="318" spans="1:8" x14ac:dyDescent="0.25">
@@ -11277,7 +11277,7 @@
         <v>14</v>
       </c>
       <c r="H318" s="1" t="s">
-        <v>146</v>
+        <v>14</v>
       </c>
     </row>
     <row r="319" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>